<commit_message>
📊 Horarios actualizados Línea 141 - 2400
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:23:34</t>
+          <t>Última actualización: 03:07:56</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:23:34</t>
+          <t>Última actualización: 03:07:56</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:23:34</t>
+          <t>Última actualización: 03:07:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2401
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:07:56</t>
+          <t>Última actualización: 04:42:04</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:07:56</t>
+          <t>Última actualización: 04:42:04</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:07:56</t>
+          <t>Última actualización: 04:42:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2402
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:42:04</t>
+          <t>Última actualización: 05:29:46</t>
         </is>
       </c>
     </row>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:42:04</t>
+          <t>Última actualización: 05:29:46</t>
         </is>
       </c>
     </row>
@@ -502,7 +502,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:42:04</t>
+          <t>Última actualización: 05:29:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2403
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,416 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:29:46</t>
+          <t>Última actualización: 06:12:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:36</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>24</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>27</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>29</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>29</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>47</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>50</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>69</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>75</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>77</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>79</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>84</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>92</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:06</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>114</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -454,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,14 +869,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:29:46</t>
+          <t>Última actualización: 06:12:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>50</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>79</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
         </is>
       </c>
     </row>
@@ -489,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,14 +1006,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:29:46</t>
+          <t>Última actualización: 06:12:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06:12:28</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>97</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2404
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:12:28</t>
+          <t>Última actualización: 07:01:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>07:02</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:02</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>75</v>
+        <v>19</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,23 +823,273 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>35</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>43</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:01</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>60</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>08:06</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>114</v>
-      </c>
-      <c r="E20" t="inlineStr">
+      <c r="D25" t="n">
+        <v>65</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>78</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>80</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>84</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>103</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>103</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -856,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -869,14 +1119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:12:28</t>
+          <t>Última actualización: 07:01:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -935,7 +1185,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -949,7 +1199,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -960,7 +1210,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:12:28</t>
+          <t>07:01:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -974,9 +1224,84 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:51</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>103</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>103</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -993,7 +1318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1006,14 +1331,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:12:28</t>
+          <t>Última actualización: 07:01:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1047,23 +1372,73 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>47</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>06:12:28</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>07:49</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>97</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07:01:39</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>96</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2405
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:39</t>
+          <t>Última actualización: 07:53:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -948,12 +948,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -978,16 +978,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:18</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1028,16 +1028,16 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>08:25</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>103</v>
+        <v>28</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,23 +1073,323 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>32</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>08:44</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>103</v>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="D31" t="n">
+        <v>51</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>51</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>08:49</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>56</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>70</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>73</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>82</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>83</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>83</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>90</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>100</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>101</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>111</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1106,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1119,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:39</t>
+          <t>Última actualización: 07:53:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1560,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1274,7 +1574,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>103</v>
+        <v>51</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1285,7 +1585,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1299,9 +1599,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>103</v>
+        <v>51</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>73</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1318,7 +1643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1331,14 +1656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:01:39</t>
+          <t>Última actualización: 07:53:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1747,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07:01:39</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1436,9 +1761,59 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>69</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>94</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2406
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:53:59</t>
+          <t>Última actualización: 08:25:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>08:49</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:49</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,12 +1223,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1253,16 +1253,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>83</v>
+        <v>70</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>90</v>
+        <v>41</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>101</v>
+        <v>82</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,18 +1378,368 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>83</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>83</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>51</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>90</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>09:24</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>59</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>100</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>69</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>101</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>70</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>09:44</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>111</v>
-      </c>
-      <c r="E42" t="inlineStr">
+      <c r="D51" t="n">
+        <v>79</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>90</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>97</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>99</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>106</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>110</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1406,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1419,14 +1769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:53:59</t>
+          <t>Última actualización: 08:25:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1910,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1574,7 +1924,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1610,23 +1960,73 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>09:06</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>73</v>
-      </c>
-      <c r="E12" t="inlineStr">
+      <c r="D13" t="n">
+        <v>41</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>90</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1643,7 +2043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1656,14 +2056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:53:59</t>
+          <t>Última actualización: 08:25:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1772,25 +2172,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09:02</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
@@ -1802,20 +2202,120 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>69</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>38</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:53:59</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>09:27</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D12" t="n">
         <v>94</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>63</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>113</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2407
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:25:21</t>
+          <t>Última actualización: 08:52:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>09:23</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,12 +1473,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>09:24</t>
+          <t>09:23</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>100</v>
+        <v>59</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,12 +1523,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>101</v>
+        <v>42</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1578,16 +1578,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>09:35</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>09:55</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>90</v>
+        <v>52</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>99</v>
+        <v>62</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,23 +1723,223 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>70</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>71</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>08:25:21</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>99</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>106</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>82</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08:25:21</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
         <is>
           <t>10:15</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="D61" t="n">
         <v>110</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>92</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>102</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>111</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1756,7 +1956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1769,14 +1969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:25:21</t>
+          <t>Última actualización: 08:52:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1985,7 +2185,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1999,7 +2199,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2010,23 +2210,48 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>62</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>08:25:21</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>09:55</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>90</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2043,7 +2268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2056,14 +2281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:25:21</t>
+          <t>Última actualización: 08:52:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2422,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2211,7 +2436,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>10</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2247,7 +2472,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2261,7 +2486,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2297,25 +2522,100 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10:17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>85</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>08:25:21</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>10:18</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>113</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>97</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:52:57</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>110</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2408
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:52:57</t>
+          <t>Última actualización: 09:34:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 69</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,7 +1623,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1723,12 +1723,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,12 +1773,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>99</v>
+        <v>71</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>106</v>
+        <v>30</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>10:14</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,12 +1848,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>10:14</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10:24</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>92</v>
+        <v>41</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:24</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>102</v>
+        <v>50</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,23 +1923,273 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>60</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>08:52:57</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D65" t="n">
         <v>111</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>70</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10:52</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>78</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>81</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>11:01</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>87</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>88</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>90</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>94</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>11:12</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>98</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>11:24</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>110</v>
+      </c>
+      <c r="E74" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1969,7 +2219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:52:57</t>
+          <t>Última actualización: 09:34:39</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2460,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2224,7 +2474,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2268,7 +2518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2281,14 +2531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:52:57</t>
+          <t>Última actualización: 09:34:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2772,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2536,7 +2786,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2572,7 +2822,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2586,7 +2836,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2597,7 +2847,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2611,11 +2861,36 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>09:34:39</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>108</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2409
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:34:39</t>
+          <t>Última actualización: 10:43:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 69</t>
+          <t>Total filas: 83</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>11:01</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>90</v>
+        <v>18</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>11:12</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>98</v>
+        <v>21</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,23 +2173,373 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>25</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
           <t>09:34:39</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11:12</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>98</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>32</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
         <is>
           <t>11:24</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D74" t="n">
-        <v>110</v>
-      </c>
-      <c r="E74" t="inlineStr">
+      <c r="D77" t="n">
+        <v>41</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>51</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>11:36</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>53</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>11:39</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>56</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>61</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>11:54</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>71</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>72</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>81</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>92</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>101</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>111</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>113</v>
+      </c>
+      <c r="E88" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2206,7 +2556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2219,14 +2569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:34:39</t>
+          <t>Última actualización: 10:43:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2502,6 +2852,56 @@
         <v>90</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>51</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>61</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2518,7 +2918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2531,14 +2931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:34:39</t>
+          <t>Última actualización: 10:43:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2872,23 +3272,48 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>10:43:47</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>10:46</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>10:43:47</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>11:22</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>108</v>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D19" t="n">
+        <v>39</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2410
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:43:47</t>
+          <t>Última actualización: 11:26:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 83</t>
+          <t>Total filas: 94</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>11:36</t>
+          <t>11:35</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>11:39</t>
+          <t>11:36</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>56</v>
+        <v>10</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2353,16 +2353,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:39</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>11:54</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:45</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>81</v>
+        <v>19</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:54</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>101</v>
+        <v>29</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>111</v>
+        <v>38</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,23 +2523,298 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>49</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
           <t>10:43:47</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>101</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>59</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>68</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
         <is>
           <t>12:36</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D88" t="n">
-        <v>113</v>
-      </c>
-      <c r="E88" t="inlineStr">
+      <c r="D92" t="n">
+        <v>70</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>78</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>78</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>12:46</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>80</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>89</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>99</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>109</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>118</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2556,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2569,14 +2844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:43:47</t>
+          <t>Última actualización: 11:26:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2885,23 +3160,98 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11:35</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>9</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>10:43:47</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>61</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>19</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>89</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2918,7 +3268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2931,14 +3281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:43:47</t>
+          <t>Última actualización: 11:26:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -3314,6 +3664,31 @@
         <v>39</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11:26:11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>117</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2411
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:26:11</t>
+          <t>Última actualización: 12:02:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 94</t>
+          <t>Total filas: 102</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>10:43:47</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>101</v>
+        <v>13</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>59</v>
+        <v>22</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>70</v>
+        <v>29</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>78</v>
+        <v>32</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2678,16 +2678,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2753,16 +2753,16 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>109</v>
+        <v>44</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,23 +2798,223 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>53</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>62</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
           <t>11:26:11</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>99</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>73</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
         <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>118</v>
-      </c>
-      <c r="E99" t="inlineStr">
+      <c r="D103" t="n">
+        <v>82</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>84</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>89</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>102</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>113</v>
+      </c>
+      <c r="E107" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2831,7 +3031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,14 +3044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:26:11</t>
+          <t>Última actualización: 12:02:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3435,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3249,9 +3449,34 @@
         </is>
       </c>
       <c r="D20" t="n">
+        <v>53</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
         <v>89</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3268,7 +3493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3281,14 +3506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:26:11</t>
+          <t>Última actualización: 12:02:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3672,7 +3897,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3686,11 +3911,36 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>12:02:23</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>108</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2412
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E107"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:02:23</t>
+          <t>Última actualización: 12:48:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 102</t>
+          <t>Total filas: 114</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:48</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,12 +2848,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>13:05</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>13:26</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>84</v>
+        <v>33</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>89</v>
+        <v>33</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3003,18 +3003,318 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
+          <t>13:26</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>84</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>43</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>56</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
           <t>13:55</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D107" t="n">
-        <v>113</v>
-      </c>
-      <c r="E107" t="inlineStr">
+      <c r="D110" t="n">
+        <v>67</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>14:04</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>76</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>83</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>86</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>86</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>88</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>96</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>103</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>107</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>14:44</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>116</v>
+      </c>
+      <c r="E119" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3031,7 +3331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3044,14 +3344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:02:23</t>
+          <t>Última actualización: 12:48:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3485,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3195,11 +3495,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -3210,7 +3510,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3220,11 +3520,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -3435,7 +3735,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3449,7 +3749,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3460,7 +3760,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3474,9 +3774,34 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>107</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3493,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3506,14 +3831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:02:23</t>
+          <t>Última actualización: 12:48:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3897,12 +4222,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3911,7 +4236,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3927,20 +4252,70 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>81</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>108</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="n">
+        <v>62</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>12:48:34</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:42</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>114</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2413
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:34</t>
+          <t>Última actualización: 13:20:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 114</t>
+          <t>Total filas: 123</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:20</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>13:26</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>13:31</t>
+          <t>13:26</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:31</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3103,16 +3103,16 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,21 +3123,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>83</v>
+        <v>25</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>14:14</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3203,16 +3203,16 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>96</v>
+        <v>54</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:14</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>103</v>
+        <v>54</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>107</v>
+        <v>88</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,23 +3298,248 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>57</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>12:48:34</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>14:24</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>96</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>65</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>14:31</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>71</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>75</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
         <is>
           <t>14:44</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D119" t="n">
-        <v>116</v>
-      </c>
-      <c r="E119" t="inlineStr">
+      <c r="D124" t="n">
+        <v>84</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>95</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>99</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>105</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>115</v>
+      </c>
+      <c r="E128" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3331,7 +3556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3344,14 +3569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:34</t>
+          <t>Última actualización: 13:20:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -3785,23 +4010,98 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>12</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>14:35</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>107</v>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D23" t="n">
+        <v>75</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>95</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>105</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3818,7 +4118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3831,14 +4131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:34</t>
+          <t>Última actualización: 13:20:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4222,12 +4522,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4236,7 +4536,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4247,12 +4547,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:22</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4261,7 +4561,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -4272,48 +4572,98 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>12:48:34</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>14:42</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>114</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>83</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2414
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:20:02</t>
+          <t>Última actualización: 13:58:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 123</t>
+          <t>Total filas: 133</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3187,7 +3187,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>83</v>
+        <v>13</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>88</v>
+        <v>18</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3337,7 +3337,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>96</v>
+        <v>26</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3373,7 +3373,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,12 +3398,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3428,16 +3428,16 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>95</v>
+        <v>46</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>99</v>
+        <v>56</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3503,16 +3503,16 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,18 +3528,268 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>99</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>63</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>66</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>105</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
           <t>15:15</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D128" t="n">
-        <v>115</v>
-      </c>
-      <c r="E128" t="inlineStr">
+      <c r="D132" t="n">
+        <v>77</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>86</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>96</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>103</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>106</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>117</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>118</v>
+      </c>
+      <c r="E138" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3556,7 +3806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3569,14 +3819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:20:02</t>
+          <t>Última actualización: 13:58:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4035,12 +4285,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4049,7 +4299,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4065,16 +4315,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4085,23 +4335,123 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>56</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>13:20:02</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>95</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>66</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:20:02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
         <is>
           <t>15:05</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="D28" t="n">
         <v>105</v>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:34</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>96</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4118,7 +4468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4131,14 +4481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:20:02</t>
+          <t>Última actualización: 13:58:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4622,7 +4972,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4636,7 +4986,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>114</v>
+        <v>44</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4666,6 +5016,31 @@
       <c r="E25" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>84</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2415
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:47</t>
+          <t>Última actualización: 14:33:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 133</t>
+          <t>Total filas: 141</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,12 +3423,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3437,7 +3437,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>14:54</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,12 +3498,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:54</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3512,7 +3512,7 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>99</v>
+        <v>22</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,12 +3548,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3562,7 +3562,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,12 +3598,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>105</v>
+        <v>66</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3703,16 +3703,16 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>117</v>
+        <v>68</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,18 +3778,218 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
+          <t>15:44</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>106</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>72</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>80</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>82</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>13:58:47</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
           <t>15:56</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C142" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D138" t="n">
+      <c r="D142" t="n">
         <v>118</v>
       </c>
-      <c r="E138" t="inlineStr">
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>84</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>91</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>101</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>111</v>
+      </c>
+      <c r="E146" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3806,7 +4006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3819,14 +4019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:47</t>
+          <t>Última actualización: 14:33:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4510,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4324,7 +4524,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4360,7 +4560,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4374,7 +4574,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>95</v>
+        <v>22</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -4410,7 +4610,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4424,7 +4624,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>105</v>
+        <v>32</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4452,6 +4652,31 @@
         <v>96</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>62</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4468,7 +4693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4481,14 +4706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:58:47</t>
+          <t>Última actualización: 14:33:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5222,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5011,7 +5236,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>83</v>
+        <v>10</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5039,6 +5264,81 @@
         <v>84</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>50</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>90</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>117</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2416
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E146"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:16</t>
+          <t>Última actualización: 15:04:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 141</t>
+          <t>Total filas: 149</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3612,7 +3612,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>42</v>
+        <v>2</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,12 +3723,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3753,16 +3753,16 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,12 +3798,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,23 +3973,223 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
+          <t>16:04</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>60</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>70</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
           <t>16:24</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
+      <c r="C148" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D146" t="n">
+      <c r="D148" t="n">
+        <v>80</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>16:34</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>90</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>91</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>97</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>16:44</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>100</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
         <v>111</v>
       </c>
-      <c r="E146" t="inlineStr">
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>117</v>
+      </c>
+      <c r="E154" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4019,7 +4219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:16</t>
+          <t>Última actualización: 15:04:41</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4785,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4599,7 +4799,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4635,7 +4835,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4649,7 +4849,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4693,7 +4893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4706,14 +4906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:16</t>
+          <t>Última actualización: 15:04:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5447,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5261,7 +5461,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5297,12 +5497,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>15:04:41</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5311,7 +5511,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5327,18 +5527,68 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>90</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>15:04:41</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>85</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:33:16</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>16:30</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D31" t="n">
         <v>117</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2417
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:04:41</t>
+          <t>Última actualización: 16:03:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 149</t>
+          <t>Total filas: 159</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3987,7 +3987,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,7 +3998,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>80</v>
+        <v>13</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,23 +4173,273 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>48</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>52</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
           <t>15:04:41</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B156" t="inlineStr">
         <is>
           <t>17:01</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C156" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D154" t="n">
+      <c r="D156" t="n">
         <v>117</v>
       </c>
-      <c r="E154" t="inlineStr">
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>61</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>71</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>81</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>87</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>92</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>93</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>101</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>111</v>
+      </c>
+      <c r="E164" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4206,7 +4456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4219,14 +4469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:04:41</t>
+          <t>Última actualización: 16:03:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4877,6 +5127,81 @@
         <v>62</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>71</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>101</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:54</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>111</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4893,7 +5218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4906,14 +5231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:04:41</t>
+          <t>Última actualización: 16:03:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5847,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5536,7 +5861,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5547,7 +5872,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>15:04:41</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5561,7 +5886,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5591,6 +5916,31 @@
       <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>79</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2418
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E164"/>
+  <dimension ref="A1:E177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:50</t>
+          <t>Última actualización: 16:47:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 159</t>
+          <t>Total filas: 172</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4303,16 +4303,16 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>92</v>
+        <v>37</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4378,16 +4378,16 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,23 +4423,348 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>48</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
           <t>16:03:50</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>93</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>50</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>101</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>58</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
         <is>
           <t>17:54</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
+      <c r="C169" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D164" t="n">
+      <c r="D169" t="n">
         <v>111</v>
       </c>
-      <c r="E164" t="inlineStr">
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>68</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>18:04</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>77</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>88</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>96</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>98</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>107</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>109</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>18:44</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>117</v>
+      </c>
+      <c r="E177" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4456,7 +4781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4469,14 +4794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:50</t>
+          <t>Última actualización: 16:47:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -5160,21 +5485,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>101</v>
+        <v>28</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5190,18 +5515,118 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>17:44</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>101</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>58</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>16:03:50</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>17:54</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D35" t="n">
         <v>111</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>68</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>88</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5218,7 +5643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5231,14 +5656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:03:50</t>
+          <t>Última actualización: 16:47:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5939,6 +6364,56 @@
         <v>79</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>36</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>16:47:09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>118</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2419
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E177"/>
+  <dimension ref="A1:E185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:09</t>
+          <t>Última actualización: 17:17:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 172</t>
+          <t>Total filas: 180</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4348,12 +4348,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>17:31</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:31</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>93</v>
+        <v>14</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>101</v>
+        <v>19</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4528,16 +4528,16 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>17:54</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4578,16 +4578,16 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>17:55</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>16:03:50</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>18:04</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>17:55</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>88</v>
+        <v>38</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4753,18 +4753,218 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>98</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>74</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>18:34</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>77</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>18:36</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>79</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
           <t>18:44</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
+      <c r="C181" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D177" t="n">
-        <v>117</v>
-      </c>
-      <c r="E177" t="inlineStr">
+      <c r="D181" t="n">
+        <v>87</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>97</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>103</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>107</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>119</v>
+      </c>
+      <c r="E185" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4781,7 +4981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4794,14 +4994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:09</t>
+          <t>Última actualización: 17:17:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5510,7 +5710,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:03:50</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5524,7 +5724,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>101</v>
+        <v>27</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5585,7 +5785,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5599,7 +5799,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5610,7 +5810,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5624,9 +5824,34 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>103</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5643,7 +5868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5656,14 +5881,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:47:09</t>
+          <t>Última actualización: 17:17:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6597,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6386,7 +6611,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6397,7 +6622,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6411,11 +6636,36 @@
         </is>
       </c>
       <c r="D34" t="n">
+        <v>88</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
         <v>118</v>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>L6203</t>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2420
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:17:28</t>
+          <t>Última actualización: 17:54:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 180</t>
+          <t>Total filas: 190</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,12 +4698,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>96</v>
+        <v>27</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>16:47:09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,12 +4748,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>16:47:09</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>18:31</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4803,16 +4803,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:31</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>18:44</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:44</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>103</v>
+        <v>51</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>107</v>
+        <v>60</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,23 +4948,273 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>66</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
           <t>17:17:28</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>107</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>71</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>19:13</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>79</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
         <is>
           <t>19:16</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>82</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>17:17:28</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D185" t="n">
+      <c r="D190" t="n">
         <v>119</v>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>83</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>90</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>91</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>115</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>19:50</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>116</v>
+      </c>
+      <c r="E195" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4981,7 +5231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4994,14 +5244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:17:28</t>
+          <t>Última actualización: 17:54:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -5785,7 +6035,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5799,7 +6049,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5810,7 +6060,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5824,7 +6074,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -5835,7 +6085,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5849,9 +6099,34 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>103</v>
+        <v>66</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>91</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5868,7 +6143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5881,14 +6156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:17:28</t>
+          <t>Última actualización: 17:54:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6897,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6636,7 +6911,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6647,7 +6922,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6661,11 +6936,36 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>118</v>
+        <v>81</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>17:54:08</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>113</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2421
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E195"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:54:08</t>
+          <t>Última actualización: 18:23:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 190</t>
+          <t>Total filas: 195</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:47</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>107</v>
+        <v>37</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,12 +4998,12 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>90</v>
+        <v>119</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>91</v>
+        <v>54</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>115</v>
+        <v>61</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,23 +5198,148 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>62</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>18:23:14</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>19:49</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>86</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>18:23:14</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
           <t>19:50</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
+      <c r="C197" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D195" t="n">
-        <v>116</v>
-      </c>
-      <c r="E195" t="inlineStr">
+      <c r="D197" t="n">
+        <v>87</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>18:23:14</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>98</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>18:23:14</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>112</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>18:23:14</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>113</v>
+      </c>
+      <c r="E200" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5231,7 +5356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5244,14 +5369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:54:08</t>
+          <t>Última actualización: 18:23:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -6085,7 +6210,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6099,7 +6224,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6110,7 +6235,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6124,9 +6249,34 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>91</v>
+        <v>62</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>18:23:14</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>112</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6156,7 +6306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:54:08</t>
+          <t>Última actualización: 18:23:14</t>
         </is>
       </c>
     </row>
@@ -6897,7 +7047,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6911,7 +7061,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6922,7 +7072,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6936,7 +7086,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6947,7 +7097,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6961,7 +7111,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2422
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:23:14</t>
+          <t>Última actualización: 18:55:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 195</t>
+          <t>Total filas: 201</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>107</v>
+        <v>5</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,12 +5023,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>71</v>
+        <v>107</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>19:11</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,12 +5073,12 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>17:54:08</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>19:13</t>
+          <t>19:11</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>79</v>
+        <v>48</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>17:54:08</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>61</v>
+        <v>119</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>86</v>
+        <v>29</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>98</v>
+        <v>54</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,23 +5323,173 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>19:56</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>61</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
           <t>18:23:14</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>98</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>20:09</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>74</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>80</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
         <is>
           <t>20:16</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
+      <c r="C204" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D200" t="n">
-        <v>113</v>
-      </c>
-      <c r="E200" t="inlineStr">
+      <c r="D204" t="n">
+        <v>81</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>105</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>107</v>
+      </c>
+      <c r="E206" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5356,7 +5506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5369,14 +5519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:23:14</t>
+          <t>Última actualización: 18:55:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6360,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6224,7 +6374,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6235,7 +6385,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6249,7 +6399,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6260,7 +6410,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6274,9 +6424,34 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>105</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6293,7 +6468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6306,14 +6481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:23:14</t>
+          <t>Última actualización: 18:55:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7247,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7086,7 +7261,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7097,7 +7272,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7111,9 +7286,34 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>104</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2423
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E206"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:55:07</t>
+          <t>Última actualización: 19:21:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 201</t>
+          <t>Total filas: 210</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5223,12 +5223,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5253,16 +5253,16 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>19:49</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>19:50</t>
+          <t>19:49</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>19:56</t>
+          <t>19:50</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,12 +5373,12 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>20:09</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5403,16 +5403,16 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:09</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>81</v>
+        <v>51</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>105</v>
+        <v>54</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,23 +5473,248 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>54</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
           <t>18:55:07</t>
         </is>
       </c>
-      <c r="B206" t="inlineStr">
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>81</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>20:36</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>75</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>78</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>18:55:07</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>105</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
         <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D206" t="n">
-        <v>107</v>
-      </c>
-      <c r="E206" t="inlineStr">
+      <c r="D211" t="n">
+        <v>81</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>92</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>95</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>104</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>106</v>
+      </c>
+      <c r="E215" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5506,7 +5731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5519,14 +5744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:55:07</t>
+          <t>Última actualización: 19:21:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5885,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5670,11 +5895,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -5685,7 +5910,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -5695,11 +5920,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -6385,7 +6610,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6399,7 +6624,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6410,7 +6635,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6424,7 +6649,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6435,23 +6660,48 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>78</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>18:55:07</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>20:40</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D42" t="n">
         <v>105</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6481,7 +6731,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:55:07</t>
+          <t>Última actualización: 19:21:32</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7522,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -7286,7 +7536,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7297,7 +7547,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7311,7 +7561,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2424
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E215"/>
+  <dimension ref="A1:E223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:32</t>
+          <t>Última actualización: 19:59:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 210</t>
+          <t>Total filas: 218</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>13:20:02</t>
+          <t>12:48:34</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12:48:34</t>
+          <t>13:20:02</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5373,12 +5373,12 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>18:23:14</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,12 +5398,12 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>18:23:14</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>20:09</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,12 +5423,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>20:12</t>
+          <t>20:09</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5453,16 +5453,16 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,12 +5473,12 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,12 +5498,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5528,16 +5528,16 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>20:40</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>105</v>
+        <v>36</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,16 +5603,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:39</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>92</v>
+        <v>40</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:40</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>104</v>
+        <v>42</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5703,18 +5703,218 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>81</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>20:53</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>54</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>57</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>66</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>21:06</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>67</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>19:21:32</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
           <t>21:07</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr">
+      <c r="C220" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D215" t="n">
+      <c r="D220" t="n">
         <v>106</v>
       </c>
-      <c r="E215" t="inlineStr">
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>95</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>96</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>97</v>
+      </c>
+      <c r="E223" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5731,7 +5931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5744,14 +5944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:32</t>
+          <t>Última actualización: 19:59:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6635,12 +6835,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6649,7 +6849,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6665,16 +6865,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>20:39</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6685,23 +6885,48 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20:39</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>40</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>18:55:07</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>20:40</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>105</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6718,7 +6943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6731,14 +6956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:21:32</t>
+          <t>Última actualización: 19:59:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7564,6 +7789,56 @@
         <v>78</v>
       </c>
       <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>42</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>19:59:58</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>21:31</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>92</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2425
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E223"/>
+  <dimension ref="A1:E228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:58</t>
+          <t>Última actualización: 20:36:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 218</t>
+          <t>Total filas: 223</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D116" t="n">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>105</v>
+        <v>4</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5723,12 +5723,12 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>20:53</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:53</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,21 +5773,21 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,12 +5823,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>106</v>
+        <v>67</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:07</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>96</v>
+        <v>58</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,23 +5898,148 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>59</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
           <t>21:36</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr">
+      <c r="C224" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D223" t="n">
-        <v>97</v>
-      </c>
-      <c r="E223" t="inlineStr">
+      <c r="D224" t="n">
+        <v>60</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>63</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>82</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>22:06</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>90</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>22:25</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>109</v>
+      </c>
+      <c r="E228" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5944,7 +6069,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:58</t>
+          <t>Última actualización: 20:36:52</t>
         </is>
       </c>
     </row>
@@ -6910,7 +7035,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6924,7 +7049,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>105</v>
+        <v>4</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -6943,7 +7068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6956,14 +7081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:58</t>
+          <t>Última actualización: 20:36:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -7822,25 +7947,75 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>20:36:52</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>14</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>21:31</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
+        <v>55</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
         <v>92</v>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>L6203</t>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 2426
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-04-12.xlsx
+++ b/data/horarios-141-2026-04-12.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E228"/>
+  <dimension ref="A1:E239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:36:52</t>
+          <t>Última actualización: 21:04:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 223</t>
+          <t>Total filas: 234</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -608,7 +608,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08:25:21</t>
+          <t>07:53:59</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07:53:59</t>
+          <t>08:25:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08:52:57</t>
+          <t>09:34:39</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>09:34:39</t>
+          <t>08:52:57</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>11:26:11</t>
+          <t>12:02:23</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>12:02:23</t>
+          <t>11:26:11</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>13:58:47</t>
+          <t>14:33:16</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3408,11 +3408,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,7 +3423,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>14:33:16</t>
+          <t>13:58:47</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3433,11 +3433,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>18:55:07</t>
+          <t>17:17:28</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>17:17:28</t>
+          <t>18:55:07</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5183,11 +5183,11 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>119</v>
+        <v>21</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>19:59:58</t>
+          <t>19:21:32</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>19:59:58</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>19:21:32</t>
+          <t>21:04:00</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>21:07</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>20:36:52</t>
+          <t>21:04:00</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:07</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>20:36:52</t>
+          <t>21:04:00</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>21:35</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:35</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>20:36:52</t>
+          <t>21:04:00</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>21:58</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>82</v>
+        <v>32</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>20:36:52</t>
+          <t>21:04:00</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>22:06</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,18 +6028,293 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
+          <t>21:39</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>63</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>21:40</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>36</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>82</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>21:59</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>55</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>22:06</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>90</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>22:07</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>63</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>20:36:52</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
           <t>22:25</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
+      <c r="C234" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D228" t="n">
+      <c r="D234" t="n">
         <v>109</v>
       </c>
-      <c r="E228" t="inlineStr">
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>83</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>93</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>22:41</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>97</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>22:51</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>107</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>22:56</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>112</v>
+      </c>
+      <c r="E239" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6056,7 +6331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6069,14 +6344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:36:52</t>
+          <t>Última actualización: 21:04:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -7052,6 +7327,31 @@
         <v>4</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>93</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7068,7 +7368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7081,14 +7381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:36:52</t>
+          <t>Última actualización: 21:04:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7997,23 +8297,73 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>21:33</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>29</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>20:36:52</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>22:08</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D41" t="n">
+      <c r="D42" t="n">
         <v>92</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>21:04:00</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>65</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>